<commit_message>
Add fitur tambah device dan printer
</commit_message>
<xml_diff>
--- a/public/assets/file/Hardware.xlsx
+++ b/public/assets/file/Hardware.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Herd\sigercep\public\assets\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1232,7 +1232,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -1249,7 +1249,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>14</v>
@@ -1300,7 +1300,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>17</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
@@ -1334,7 +1334,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>21</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>23</v>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>26</v>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>28</v>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>30</v>
@@ -1419,7 +1419,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>32</v>
@@ -1436,7 +1436,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>35</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>37</v>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>39</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>41</v>
@@ -1504,7 +1504,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>43</v>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>45</v>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>47</v>
@@ -1555,7 +1555,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>49</v>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>52</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>54</v>
@@ -1606,7 +1606,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>57</v>
@@ -1623,7 +1623,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>59</v>
@@ -1640,7 +1640,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>61</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>63</v>
@@ -1674,7 +1674,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>65</v>
@@ -1691,7 +1691,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>68</v>
@@ -1708,7 +1708,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>70</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>72</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>74</v>
@@ -1759,7 +1759,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>76</v>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>78</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>80</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>82</v>
@@ -1827,7 +1827,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>15</v>
@@ -1844,7 +1844,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>85</v>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>87</v>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>89</v>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>91</v>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>94</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>96</v>
@@ -1946,7 +1946,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>98</v>
@@ -1963,7 +1963,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>100</v>
@@ -1980,7 +1980,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>102</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>104</v>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>106</v>
@@ -2031,7 +2031,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>108</v>
@@ -2048,7 +2048,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>110</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>112</v>
@@ -2082,7 +2082,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>114</v>
@@ -2099,7 +2099,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>116</v>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>118</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>120</v>
@@ -2150,7 +2150,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>122</v>
@@ -2167,7 +2167,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>124</v>
@@ -2184,7 +2184,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>126</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>128</v>
@@ -2218,7 +2218,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>130</v>
@@ -2235,7 +2235,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>132</v>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>134</v>
@@ -2269,7 +2269,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>136</v>
@@ -2286,7 +2286,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>138</v>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>140</v>
@@ -2320,7 +2320,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>142</v>
@@ -2337,7 +2337,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>145</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>147</v>
@@ -2371,7 +2371,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>149</v>
@@ -2388,7 +2388,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>151</v>
@@ -2405,7 +2405,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>153</v>
@@ -2422,7 +2422,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>155</v>
@@ -2439,7 +2439,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>158</v>
@@ -2456,7 +2456,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>160</v>
@@ -2473,7 +2473,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>163</v>
@@ -2490,7 +2490,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>165</v>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>167</v>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>170</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>172</v>
@@ -2558,7 +2558,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>174</v>
@@ -2575,7 +2575,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>176</v>
@@ -2592,7 +2592,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>179</v>
@@ -2609,7 +2609,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>181</v>
@@ -2626,7 +2626,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>184</v>
@@ -2643,7 +2643,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>186</v>
@@ -2660,7 +2660,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>189</v>
@@ -2677,7 +2677,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>191</v>
@@ -2694,7 +2694,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>193</v>
@@ -2711,7 +2711,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>195</v>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>197</v>
@@ -2745,7 +2745,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>199</v>
@@ -2762,7 +2762,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>201</v>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>203</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>205</v>
@@ -2813,7 +2813,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>207</v>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>209</v>
@@ -2847,7 +2847,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>211</v>
@@ -2864,7 +2864,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>213</v>
@@ -2881,7 +2881,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>215</v>
@@ -2898,7 +2898,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>218</v>
@@ -2915,7 +2915,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>220</v>
@@ -2932,7 +2932,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>221</v>
@@ -2949,7 +2949,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>223</v>
@@ -2966,7 +2966,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>226</v>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>228</v>
@@ -3000,7 +3000,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>230</v>
@@ -3017,7 +3017,7 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>232</v>
@@ -3034,7 +3034,7 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>234</v>
@@ -3051,7 +3051,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>236</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
         <v>238</v>
@@ -3085,7 +3085,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>240</v>
@@ -3102,7 +3102,7 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>243</v>
@@ -3119,7 +3119,7 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>245</v>
@@ -3136,7 +3136,7 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>247</v>
@@ -3153,7 +3153,7 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>249</v>
@@ -3170,7 +3170,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>251</v>
@@ -3187,7 +3187,7 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>253</v>
@@ -3204,7 +3204,7 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>255</v>
@@ -3221,7 +3221,7 @@
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>257</v>
@@ -3238,7 +3238,7 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>259</v>

</xml_diff>

<commit_message>
fix perubahan device dan printer
</commit_message>
<xml_diff>
--- a/public/assets/file/Hardware.xlsx
+++ b/public/assets/file/Hardware.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="267">
   <si>
     <t>No</t>
   </si>
@@ -42,784 +42,784 @@
     <t>Admisi dan Billing</t>
   </si>
   <si>
+    <t>Admisi Ranap 1</t>
+  </si>
+  <si>
+    <t>Billing 2</t>
+  </si>
+  <si>
+    <t>Billing 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Service </t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>192.168.111.125</t>
+  </si>
+  <si>
+    <t>PIC ADMISI</t>
+  </si>
+  <si>
+    <t>192.168.111.141</t>
+  </si>
+  <si>
+    <t>PIPP</t>
+  </si>
+  <si>
+    <t>192.168.111.142</t>
+  </si>
+  <si>
+    <t>Operator</t>
+  </si>
+  <si>
+    <t>192.168.111.145</t>
+  </si>
+  <si>
+    <t>Rekam Medis Luar 1</t>
+  </si>
+  <si>
+    <t>Rekam Medis</t>
+  </si>
+  <si>
+    <t>192.168.111.127</t>
+  </si>
+  <si>
+    <t>Rekam Medis Luar 2</t>
+  </si>
+  <si>
+    <t>192.168.111.122</t>
+  </si>
+  <si>
+    <t>Rekam Medis Dalam 1</t>
+  </si>
+  <si>
+    <t>192.168.111.120</t>
+  </si>
+  <si>
+    <t>Rekam Medis Dalam 2</t>
+  </si>
+  <si>
+    <t>192.168.111.121</t>
+  </si>
+  <si>
+    <t>Farmasi Layanan Ranap</t>
+  </si>
+  <si>
+    <t>Farmasi</t>
+  </si>
+  <si>
+    <t>192.168.111.136</t>
+  </si>
+  <si>
+    <t>Farmasi Layanan 1</t>
+  </si>
+  <si>
+    <t>192.168.111.137</t>
+  </si>
+  <si>
+    <t>Farmasi Layanan 2</t>
+  </si>
+  <si>
+    <t>192.168.111.138</t>
+  </si>
+  <si>
+    <t>Farmasi Pemberkasan 2</t>
+  </si>
+  <si>
+    <t>Farmasi Pemberkasan 1</t>
+  </si>
+  <si>
+    <t>Farmasi Gudang 1</t>
+  </si>
+  <si>
+    <t>192.168.111.129</t>
+  </si>
+  <si>
+    <t>Farmasi Gudang 2</t>
+  </si>
+  <si>
+    <t>192.168.111.131</t>
+  </si>
+  <si>
+    <t>Farmasi Gudang 3</t>
+  </si>
+  <si>
+    <t>192.168.111.130</t>
+  </si>
+  <si>
+    <t>Gizi 1</t>
+  </si>
+  <si>
+    <t>Gizi</t>
+  </si>
+  <si>
+    <t>192.168.115.122</t>
+  </si>
+  <si>
+    <t>Gizi 2</t>
+  </si>
+  <si>
+    <t>192.168.115.121</t>
+  </si>
+  <si>
+    <t>Pengadaan Umum</t>
+  </si>
+  <si>
+    <t>Gudang</t>
+  </si>
+  <si>
+    <t>192.168.115.136</t>
+  </si>
+  <si>
+    <t>Kesehatan Lingkungan</t>
+  </si>
+  <si>
+    <t>192.168.115.131</t>
+  </si>
+  <si>
+    <t>Koor. Pemeliharaan</t>
+  </si>
+  <si>
+    <t>192.168.115.130</t>
+  </si>
+  <si>
+    <t>Atem</t>
+  </si>
+  <si>
+    <t>192.168.115.134</t>
+  </si>
+  <si>
+    <t>Bimroh</t>
+  </si>
+  <si>
+    <t>192.168.115.133</t>
+  </si>
+  <si>
+    <t>Nurse Station UGD 1</t>
+  </si>
+  <si>
+    <t>UGD</t>
+  </si>
+  <si>
+    <t>192.168.113.126</t>
+  </si>
+  <si>
+    <t>Nurse Station UGD 2</t>
+  </si>
+  <si>
+    <t>192.168.113.128</t>
+  </si>
+  <si>
+    <t>Nurse Station UGD 3</t>
+  </si>
+  <si>
+    <t>192.168.113.127</t>
+  </si>
+  <si>
+    <t>KI UGD</t>
+  </si>
+  <si>
+    <t>192.168.113.129</t>
+  </si>
+  <si>
+    <t>Admisi UGD 1</t>
+  </si>
+  <si>
+    <t>192.168.113.123</t>
+  </si>
+  <si>
+    <t>Farmasi UGD</t>
+  </si>
+  <si>
+    <t>192.168.113.122</t>
+  </si>
+  <si>
+    <t>SPV Layanan Pelanggan</t>
+  </si>
+  <si>
+    <t>192.168.113.121</t>
+  </si>
+  <si>
+    <t>SPV Pemasaran</t>
+  </si>
+  <si>
+    <t>192.168.113.119</t>
+  </si>
+  <si>
+    <t>Penjualan</t>
+  </si>
+  <si>
+    <t>192.168.113.117</t>
+  </si>
+  <si>
+    <t>192.168.113.120</t>
+  </si>
+  <si>
+    <t>Desain Grafis</t>
+  </si>
+  <si>
+    <t>192.168.113.118</t>
+  </si>
+  <si>
+    <t>MCU</t>
+  </si>
+  <si>
+    <t>192.168.121.125</t>
+  </si>
+  <si>
+    <t>NS Fisioterapi</t>
+  </si>
+  <si>
+    <t>10.10.153.54</t>
+  </si>
+  <si>
+    <t>Dokter Rehab Medik</t>
+  </si>
+  <si>
+    <t>Dokter</t>
+  </si>
+  <si>
+    <t>192.168.121.129</t>
+  </si>
+  <si>
+    <t>Admisi Rajal BPJS 1</t>
+  </si>
+  <si>
+    <t>192.168.121.141</t>
+  </si>
+  <si>
+    <t>Admisi Rajal BPJS 2</t>
+  </si>
+  <si>
+    <t>192.168.121.140</t>
+  </si>
+  <si>
+    <t>Admisi Rajal BPJS 3</t>
+  </si>
+  <si>
+    <t>192.168.121.136</t>
+  </si>
+  <si>
+    <t>Nurse Station Poli 1</t>
+  </si>
+  <si>
+    <t>192.168.123.121</t>
+  </si>
+  <si>
+    <t>Nurse Station Poli 2</t>
+  </si>
+  <si>
+    <t>192.168.123.122</t>
+  </si>
+  <si>
+    <t>Nurse Station Poli 3</t>
+  </si>
+  <si>
+    <t>192.168.123.123</t>
+  </si>
+  <si>
+    <t>Nurse Station Poli 4</t>
+  </si>
+  <si>
+    <t>192.168.123.120</t>
+  </si>
+  <si>
+    <t>Nurse Station Poli Ibu dan Anak</t>
+  </si>
+  <si>
+    <t>192.168.123.124</t>
+  </si>
+  <si>
+    <t>Dokter Poli 1</t>
+  </si>
+  <si>
+    <t>192.168.123.153</t>
+  </si>
+  <si>
+    <t>Dokter Poli 2</t>
+  </si>
+  <si>
+    <t>192.168.123.155</t>
+  </si>
+  <si>
+    <t>Dokter Poli 3</t>
+  </si>
+  <si>
+    <t>192.168.123.151</t>
+  </si>
+  <si>
+    <t>Dokter Poli 4</t>
+  </si>
+  <si>
+    <t>192.168.123.149</t>
+  </si>
+  <si>
+    <t>Dokter Poli 5</t>
+  </si>
+  <si>
+    <t>192.168.123.128</t>
+  </si>
+  <si>
+    <t>Dokter Poli 6</t>
+  </si>
+  <si>
+    <t>192.168.123.129</t>
+  </si>
+  <si>
+    <t>Dokter Poli 7</t>
+  </si>
+  <si>
+    <t>192.168.123.147</t>
+  </si>
+  <si>
+    <t>Dokter Poli 8</t>
+  </si>
+  <si>
+    <t>192.168.123.145</t>
+  </si>
+  <si>
+    <t>Dokter Poli 9</t>
+  </si>
+  <si>
+    <t>192.168.123.143</t>
+  </si>
+  <si>
+    <t>Dokter Poli 10</t>
+  </si>
+  <si>
+    <t>192.168.123.141</t>
+  </si>
+  <si>
+    <t>Dokter Poli 11</t>
+  </si>
+  <si>
+    <t>192.168.123.139</t>
+  </si>
+  <si>
+    <t>Dokter Poli 12</t>
+  </si>
+  <si>
+    <t>192.168.123.137</t>
+  </si>
+  <si>
+    <t>Dokter Poli 13</t>
+  </si>
+  <si>
+    <t>192.168.123.135</t>
+  </si>
+  <si>
+    <t>Dokter Poli 14</t>
+  </si>
+  <si>
+    <t>192.168.123.134</t>
+  </si>
+  <si>
+    <t>Dokter Poli 15</t>
+  </si>
+  <si>
+    <t>192.168.125.129</t>
+  </si>
+  <si>
+    <t>Dokter Poli 16</t>
+  </si>
+  <si>
+    <t>192.168.125.142</t>
+  </si>
+  <si>
+    <t>Nurse Station Laboratorium 1</t>
+  </si>
+  <si>
+    <t>Laboratorium</t>
+  </si>
+  <si>
+    <t>192.168.127.122</t>
+  </si>
+  <si>
+    <t>Nurse Station Laboratorium 2</t>
+  </si>
+  <si>
+    <t>192.168.127.121</t>
+  </si>
+  <si>
+    <t>Laboratorium Patologi Anatomi</t>
+  </si>
+  <si>
+    <t>192.168.127.132</t>
+  </si>
+  <si>
+    <t>Bank Darah</t>
+  </si>
+  <si>
+    <t>192.168.127.126</t>
+  </si>
+  <si>
+    <t>KI Lab</t>
+  </si>
+  <si>
+    <t>192.168.127.129</t>
+  </si>
+  <si>
+    <t>Laboratorium Analitik</t>
+  </si>
+  <si>
+    <t>192.168.127.138</t>
+  </si>
+  <si>
+    <t>NS Hemodialisa</t>
+  </si>
+  <si>
+    <t>HD</t>
+  </si>
+  <si>
+    <t>192.168.125.136</t>
+  </si>
+  <si>
+    <t>Admisi Hemodialisa</t>
+  </si>
+  <si>
+    <t>192.168.125.137</t>
+  </si>
+  <si>
+    <t>Admisi Radiologi</t>
+  </si>
+  <si>
+    <t>Radiologi</t>
+  </si>
+  <si>
+    <t>192.168.125.138</t>
+  </si>
+  <si>
+    <t>Dokter Radiologi</t>
+  </si>
+  <si>
+    <t>192.168.125.133</t>
+  </si>
+  <si>
+    <t>Dokter OK</t>
+  </si>
+  <si>
+    <t>192.168.131.122</t>
+  </si>
+  <si>
+    <t>Admin OK</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>192.168.131.121</t>
+  </si>
+  <si>
+    <t>KI OK</t>
+  </si>
+  <si>
+    <t>192.168.131.126</t>
+  </si>
+  <si>
+    <t>Depo Farmasi OK</t>
+  </si>
+  <si>
+    <t>192.168.131.123</t>
+  </si>
+  <si>
+    <t>CSSD</t>
+  </si>
+  <si>
+    <t>192.168.131.125</t>
+  </si>
+  <si>
+    <t>Nurstation ICU 2</t>
+  </si>
+  <si>
+    <t>ICU</t>
+  </si>
+  <si>
+    <t>Nurstation ICU 1</t>
+  </si>
+  <si>
+    <t>NS NICU</t>
+  </si>
+  <si>
+    <t>NICU dan PICU</t>
+  </si>
+  <si>
+    <t>192.168.135.125</t>
+  </si>
+  <si>
+    <t>NS PICU</t>
+  </si>
+  <si>
+    <t>192.168.135.124</t>
+  </si>
+  <si>
+    <t>NS Ruang Permata</t>
+  </si>
+  <si>
+    <t>Perawat</t>
+  </si>
+  <si>
+    <t>192.168.135.120</t>
+  </si>
+  <si>
+    <t>Nurstation VK 1</t>
+  </si>
+  <si>
+    <t>192.168.133.143</t>
+  </si>
+  <si>
+    <t>Nurstation VK 2</t>
+  </si>
+  <si>
+    <t>192.168.133.142</t>
+  </si>
+  <si>
+    <t>Staff Keuangan Anissa</t>
+  </si>
+  <si>
+    <t>192.168.141.16</t>
+  </si>
+  <si>
+    <t>Staff Keuangan Ainun</t>
+  </si>
+  <si>
+    <t>192.168.141.128</t>
+  </si>
+  <si>
+    <t>Staff Keuangan Wira</t>
+  </si>
+  <si>
+    <t>192.168.141.129</t>
+  </si>
+  <si>
+    <t>Staff Keuangan Viola</t>
+  </si>
+  <si>
+    <t>192.168.141.137</t>
+  </si>
+  <si>
+    <t>Staff Akuntansi Rika</t>
+  </si>
+  <si>
+    <t>192.168.141.125</t>
+  </si>
+  <si>
+    <t>Staff Akuntansi Evi</t>
+  </si>
+  <si>
+    <t>192.168.141.124</t>
+  </si>
+  <si>
+    <t>Staff Bendahara Syifa</t>
+  </si>
+  <si>
+    <t>192.168.141.132</t>
+  </si>
+  <si>
+    <t>Staff Akuntansi Dian</t>
+  </si>
+  <si>
+    <t>192.168.141.122</t>
+  </si>
+  <si>
+    <t>Staff Mutu</t>
+  </si>
+  <si>
+    <t>192.168.141.121</t>
+  </si>
+  <si>
+    <t>PPI</t>
+  </si>
+  <si>
+    <t>192.168.141.136</t>
+  </si>
+  <si>
+    <t>SPV Perawat Pak Rizal</t>
+  </si>
+  <si>
+    <t>192.168.141.135</t>
+  </si>
+  <si>
+    <t>SPV Legal</t>
+  </si>
+  <si>
+    <t>SDM</t>
+  </si>
+  <si>
+    <t>192.168.141.133</t>
+  </si>
+  <si>
+    <t>Staff Diklat dan Pengembangan</t>
+  </si>
+  <si>
+    <t>192.168.141.131</t>
+  </si>
+  <si>
+    <t>Staff SDM Aldi</t>
+  </si>
+  <si>
+    <t>Staff Legal Fajar</t>
+  </si>
+  <si>
+    <t>192.168.141.130</t>
+  </si>
+  <si>
+    <t>SPV Teknologi Informasi</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>192.168.142.20</t>
+  </si>
+  <si>
+    <t>Pengembangan Sistem Novit</t>
+  </si>
+  <si>
+    <t>192.168.142.88</t>
+  </si>
+  <si>
+    <t>Infrastruktur Iyan</t>
+  </si>
+  <si>
+    <t>192.168.142.12</t>
+  </si>
+  <si>
+    <t>Operasional IT Ibnu</t>
+  </si>
+  <si>
+    <t>192.168.142.22</t>
+  </si>
+  <si>
+    <t>Operasional IT Samuel</t>
+  </si>
+  <si>
+    <t>192.168.142.33</t>
+  </si>
+  <si>
+    <t>Nurstation Lt4 1</t>
+  </si>
+  <si>
+    <t>192.168.143.121</t>
+  </si>
+  <si>
+    <t>Nurstation Lt4 2</t>
+  </si>
+  <si>
+    <t>192.168.143.120</t>
+  </si>
+  <si>
+    <t>KI Ranap</t>
+  </si>
+  <si>
+    <t>192.168.143.126</t>
+  </si>
+  <si>
+    <t>Staff Casemix Via</t>
+  </si>
+  <si>
+    <t>Casemix</t>
+  </si>
+  <si>
+    <t>192.168.151.139</t>
+  </si>
+  <si>
+    <t>Staff Casemix Ranti</t>
+  </si>
+  <si>
+    <t>192.168.151.137</t>
+  </si>
+  <si>
+    <t>Staff Casemix Noval</t>
+  </si>
+  <si>
+    <t>192.168.151.140</t>
+  </si>
+  <si>
+    <t>Staff Casemix Adi</t>
+  </si>
+  <si>
+    <t>192.168.151.141</t>
+  </si>
+  <si>
+    <t>Staff Casemix Ryan</t>
+  </si>
+  <si>
+    <t>192.168.151.136</t>
+  </si>
+  <si>
+    <t>Staff Casemix Yudha</t>
+  </si>
+  <si>
+    <t>192.168.151.142</t>
+  </si>
+  <si>
+    <t>Staff Casemix Wahyu</t>
+  </si>
+  <si>
+    <t>192.168.151.143</t>
+  </si>
+  <si>
+    <t>Nurstation Lt5 1</t>
+  </si>
+  <si>
+    <t>192.168.151.121</t>
+  </si>
+  <si>
+    <t>Nurstation Lt5 2</t>
+  </si>
+  <si>
+    <t>192.168.151.120</t>
+  </si>
+  <si>
+    <t>Nurstation Lt5 3</t>
+  </si>
+  <si>
+    <t>192.168.151.122</t>
+  </si>
+  <si>
+    <t>Fisioterapi</t>
+  </si>
+  <si>
+    <t>192.168.141.134</t>
+  </si>
+  <si>
+    <t>IPSRS</t>
+  </si>
+  <si>
+    <t>Poli</t>
+  </si>
+  <si>
+    <t>Keuangan &amp; Akuntansi</t>
+  </si>
+  <si>
+    <t>Komite</t>
+  </si>
+  <si>
+    <t>Gudang Umum</t>
+  </si>
+  <si>
+    <t>10.10.152.223</t>
+  </si>
+  <si>
+    <t>192.168.111.123</t>
+  </si>
+  <si>
     <t>192.168.111.124</t>
   </si>
   <si>
-    <t>Admisi Ranap 1</t>
-  </si>
-  <si>
-    <t>192.168.111.123</t>
-  </si>
-  <si>
-    <t>Billing 2</t>
+    <t>192.168.111.146</t>
   </si>
   <si>
     <t>192.168.111.140</t>
   </si>
   <si>
-    <t>Billing 1</t>
-  </si>
-  <si>
-    <t>192.168.111.146</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer Service </t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>192.168.111.125</t>
-  </si>
-  <si>
-    <t>PIC ADMISI</t>
-  </si>
-  <si>
-    <t>192.168.111.141</t>
-  </si>
-  <si>
-    <t>PIPP</t>
-  </si>
-  <si>
-    <t>192.168.111.142</t>
-  </si>
-  <si>
-    <t>Operator</t>
-  </si>
-  <si>
-    <t>192.168.111.145</t>
-  </si>
-  <si>
-    <t>Rekam Medis Luar 1</t>
-  </si>
-  <si>
-    <t>Rekam Medis</t>
-  </si>
-  <si>
-    <t>192.168.111.127</t>
-  </si>
-  <si>
-    <t>Rekam Medis Luar 2</t>
-  </si>
-  <si>
-    <t>192.168.111.122</t>
-  </si>
-  <si>
-    <t>Rekam Medis Dalam 1</t>
-  </si>
-  <si>
-    <t>192.168.111.120</t>
-  </si>
-  <si>
-    <t>Rekam Medis Dalam 2</t>
-  </si>
-  <si>
-    <t>192.168.111.121</t>
-  </si>
-  <si>
-    <t>Farmasi Layanan Ranap</t>
-  </si>
-  <si>
-    <t>Farmasi</t>
-  </si>
-  <si>
-    <t>192.168.111.136</t>
-  </si>
-  <si>
-    <t>Farmasi Layanan 1</t>
-  </si>
-  <si>
-    <t>192.168.111.137</t>
-  </si>
-  <si>
-    <t>Farmasi Layanan 2</t>
-  </si>
-  <si>
-    <t>192.168.111.138</t>
-  </si>
-  <si>
-    <t>Farmasi Pemberkasan 2</t>
+    <t>192.168.111.132</t>
   </si>
   <si>
     <t>192.168.111.134</t>
-  </si>
-  <si>
-    <t>Farmasi Pemberkasan 1</t>
-  </si>
-  <si>
-    <t>192.168.111.132</t>
-  </si>
-  <si>
-    <t>Farmasi Gudang 1</t>
-  </si>
-  <si>
-    <t>192.168.111.129</t>
-  </si>
-  <si>
-    <t>Farmasi Gudang 2</t>
-  </si>
-  <si>
-    <t>192.168.111.131</t>
-  </si>
-  <si>
-    <t>Farmasi Gudang 3</t>
-  </si>
-  <si>
-    <t>192.168.111.130</t>
-  </si>
-  <si>
-    <t>Gizi 1</t>
-  </si>
-  <si>
-    <t>Gizi</t>
-  </si>
-  <si>
-    <t>192.168.115.122</t>
-  </si>
-  <si>
-    <t>Gizi 2</t>
-  </si>
-  <si>
-    <t>192.168.115.121</t>
-  </si>
-  <si>
-    <t>Pengadaan Umum</t>
-  </si>
-  <si>
-    <t>Gudang</t>
-  </si>
-  <si>
-    <t>192.168.115.136</t>
-  </si>
-  <si>
-    <t>Kesehatan Lingkungan</t>
-  </si>
-  <si>
-    <t>192.168.115.131</t>
-  </si>
-  <si>
-    <t>Koor. Pemeliharaan</t>
-  </si>
-  <si>
-    <t>192.168.115.130</t>
-  </si>
-  <si>
-    <t>Atem</t>
-  </si>
-  <si>
-    <t>192.168.115.134</t>
-  </si>
-  <si>
-    <t>Bimroh</t>
-  </si>
-  <si>
-    <t>192.168.115.133</t>
-  </si>
-  <si>
-    <t>Nurse Station UGD 1</t>
-  </si>
-  <si>
-    <t>UGD</t>
-  </si>
-  <si>
-    <t>192.168.113.126</t>
-  </si>
-  <si>
-    <t>Nurse Station UGD 2</t>
-  </si>
-  <si>
-    <t>192.168.113.128</t>
-  </si>
-  <si>
-    <t>Nurse Station UGD 3</t>
-  </si>
-  <si>
-    <t>192.168.113.127</t>
-  </si>
-  <si>
-    <t>KI UGD</t>
-  </si>
-  <si>
-    <t>192.168.113.129</t>
-  </si>
-  <si>
-    <t>Admisi UGD 1</t>
-  </si>
-  <si>
-    <t>192.168.113.123</t>
-  </si>
-  <si>
-    <t>Farmasi UGD</t>
-  </si>
-  <si>
-    <t>192.168.113.122</t>
-  </si>
-  <si>
-    <t>SPV Layanan Pelanggan</t>
-  </si>
-  <si>
-    <t>192.168.113.121</t>
-  </si>
-  <si>
-    <t>SPV Pemasaran</t>
-  </si>
-  <si>
-    <t>192.168.113.119</t>
-  </si>
-  <si>
-    <t>Penjualan</t>
-  </si>
-  <si>
-    <t>192.168.113.117</t>
-  </si>
-  <si>
-    <t>192.168.113.120</t>
-  </si>
-  <si>
-    <t>Desain Grafis</t>
-  </si>
-  <si>
-    <t>192.168.113.118</t>
-  </si>
-  <si>
-    <t>MCU</t>
-  </si>
-  <si>
-    <t>192.168.121.125</t>
-  </si>
-  <si>
-    <t>NS Fisioterapi</t>
-  </si>
-  <si>
-    <t>10.10.153.54</t>
-  </si>
-  <si>
-    <t>Dokter Rehab Medik</t>
-  </si>
-  <si>
-    <t>Dokter</t>
-  </si>
-  <si>
-    <t>192.168.121.129</t>
-  </si>
-  <si>
-    <t>Admisi Rajal BPJS 1</t>
-  </si>
-  <si>
-    <t>192.168.121.141</t>
-  </si>
-  <si>
-    <t>Admisi Rajal BPJS 2</t>
-  </si>
-  <si>
-    <t>192.168.121.140</t>
-  </si>
-  <si>
-    <t>Admisi Rajal BPJS 3</t>
-  </si>
-  <si>
-    <t>192.168.121.136</t>
-  </si>
-  <si>
-    <t>Nurse Station Poli 1</t>
-  </si>
-  <si>
-    <t>192.168.123.121</t>
-  </si>
-  <si>
-    <t>Nurse Station Poli 2</t>
-  </si>
-  <si>
-    <t>192.168.123.122</t>
-  </si>
-  <si>
-    <t>Nurse Station Poli 3</t>
-  </si>
-  <si>
-    <t>192.168.123.123</t>
-  </si>
-  <si>
-    <t>Nurse Station Poli 4</t>
-  </si>
-  <si>
-    <t>192.168.123.120</t>
-  </si>
-  <si>
-    <t>Nurse Station Poli Ibu dan Anak</t>
-  </si>
-  <si>
-    <t>192.168.123.124</t>
-  </si>
-  <si>
-    <t>Dokter Poli 1</t>
-  </si>
-  <si>
-    <t>192.168.123.153</t>
-  </si>
-  <si>
-    <t>Dokter Poli 2</t>
-  </si>
-  <si>
-    <t>192.168.123.155</t>
-  </si>
-  <si>
-    <t>Dokter Poli 3</t>
-  </si>
-  <si>
-    <t>192.168.123.151</t>
-  </si>
-  <si>
-    <t>Dokter Poli 4</t>
-  </si>
-  <si>
-    <t>192.168.123.149</t>
-  </si>
-  <si>
-    <t>Dokter Poli 5</t>
-  </si>
-  <si>
-    <t>192.168.123.128</t>
-  </si>
-  <si>
-    <t>Dokter Poli 6</t>
-  </si>
-  <si>
-    <t>192.168.123.129</t>
-  </si>
-  <si>
-    <t>Dokter Poli 7</t>
-  </si>
-  <si>
-    <t>192.168.123.147</t>
-  </si>
-  <si>
-    <t>Dokter Poli 8</t>
-  </si>
-  <si>
-    <t>192.168.123.145</t>
-  </si>
-  <si>
-    <t>Dokter Poli 9</t>
-  </si>
-  <si>
-    <t>192.168.123.143</t>
-  </si>
-  <si>
-    <t>Dokter Poli 10</t>
-  </si>
-  <si>
-    <t>192.168.123.141</t>
-  </si>
-  <si>
-    <t>Dokter Poli 11</t>
-  </si>
-  <si>
-    <t>192.168.123.139</t>
-  </si>
-  <si>
-    <t>Dokter Poli 12</t>
-  </si>
-  <si>
-    <t>192.168.123.137</t>
-  </si>
-  <si>
-    <t>Dokter Poli 13</t>
-  </si>
-  <si>
-    <t>192.168.123.135</t>
-  </si>
-  <si>
-    <t>Dokter Poli 14</t>
-  </si>
-  <si>
-    <t>192.168.123.134</t>
-  </si>
-  <si>
-    <t>Dokter Poli 15</t>
-  </si>
-  <si>
-    <t>192.168.125.129</t>
-  </si>
-  <si>
-    <t>Dokter Poli 16</t>
-  </si>
-  <si>
-    <t>192.168.125.142</t>
-  </si>
-  <si>
-    <t>Nurse Station Laboratorium 1</t>
-  </si>
-  <si>
-    <t>Laboratorium</t>
-  </si>
-  <si>
-    <t>192.168.127.122</t>
-  </si>
-  <si>
-    <t>Nurse Station Laboratorium 2</t>
-  </si>
-  <si>
-    <t>192.168.127.121</t>
-  </si>
-  <si>
-    <t>Laboratorium Patologi Anatomi</t>
-  </si>
-  <si>
-    <t>192.168.127.132</t>
-  </si>
-  <si>
-    <t>Bank Darah</t>
-  </si>
-  <si>
-    <t>192.168.127.126</t>
-  </si>
-  <si>
-    <t>KI Lab</t>
-  </si>
-  <si>
-    <t>192.168.127.129</t>
-  </si>
-  <si>
-    <t>Laboratorium Analitik</t>
-  </si>
-  <si>
-    <t>192.168.127.138</t>
-  </si>
-  <si>
-    <t>NS Hemodialisa</t>
-  </si>
-  <si>
-    <t>HD</t>
-  </si>
-  <si>
-    <t>192.168.125.136</t>
-  </si>
-  <si>
-    <t>Admisi Hemodialisa</t>
-  </si>
-  <si>
-    <t>192.168.125.137</t>
-  </si>
-  <si>
-    <t>Admisi Radiologi</t>
-  </si>
-  <si>
-    <t>Radiologi</t>
-  </si>
-  <si>
-    <t>192.168.125.138</t>
-  </si>
-  <si>
-    <t>Dokter Radiologi</t>
-  </si>
-  <si>
-    <t>192.168.125.133</t>
-  </si>
-  <si>
-    <t>Dokter OK</t>
-  </si>
-  <si>
-    <t>192.168.131.122</t>
-  </si>
-  <si>
-    <t>Admin OK</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>192.168.131.121</t>
-  </si>
-  <si>
-    <t>KI OK</t>
-  </si>
-  <si>
-    <t>192.168.131.126</t>
-  </si>
-  <si>
-    <t>Depo Farmasi OK</t>
-  </si>
-  <si>
-    <t>192.168.131.123</t>
-  </si>
-  <si>
-    <t>CSSD</t>
-  </si>
-  <si>
-    <t>192.168.131.125</t>
-  </si>
-  <si>
-    <t>Nurstation ICU 2</t>
-  </si>
-  <si>
-    <t>ICU</t>
-  </si>
-  <si>
-    <t>192.168.133.121</t>
-  </si>
-  <si>
-    <t>Nurstation ICU 1</t>
-  </si>
-  <si>
-    <t>192.168.133.120</t>
-  </si>
-  <si>
-    <t>NS NICU</t>
-  </si>
-  <si>
-    <t>NICU dan PICU</t>
-  </si>
-  <si>
-    <t>192.168.135.125</t>
-  </si>
-  <si>
-    <t>NS PICU</t>
-  </si>
-  <si>
-    <t>192.168.135.124</t>
-  </si>
-  <si>
-    <t>NS Ruang Permata</t>
-  </si>
-  <si>
-    <t>Perawat</t>
-  </si>
-  <si>
-    <t>192.168.135.120</t>
-  </si>
-  <si>
-    <t>Nurstation VK 1</t>
-  </si>
-  <si>
-    <t>192.168.133.143</t>
-  </si>
-  <si>
-    <t>Nurstation VK 2</t>
-  </si>
-  <si>
-    <t>192.168.133.142</t>
-  </si>
-  <si>
-    <t>Staff Keuangan Anissa</t>
-  </si>
-  <si>
-    <t>192.168.141.16</t>
-  </si>
-  <si>
-    <t>Staff Keuangan Ainun</t>
-  </si>
-  <si>
-    <t>192.168.141.128</t>
-  </si>
-  <si>
-    <t>Staff Keuangan Wira</t>
-  </si>
-  <si>
-    <t>192.168.141.129</t>
-  </si>
-  <si>
-    <t>Staff Keuangan Viola</t>
-  </si>
-  <si>
-    <t>192.168.141.137</t>
-  </si>
-  <si>
-    <t>Staff Akuntansi Rika</t>
-  </si>
-  <si>
-    <t>192.168.141.125</t>
-  </si>
-  <si>
-    <t>Staff Akuntansi Evi</t>
-  </si>
-  <si>
-    <t>192.168.141.124</t>
-  </si>
-  <si>
-    <t>Staff Bendahara Syifa</t>
-  </si>
-  <si>
-    <t>192.168.141.132</t>
-  </si>
-  <si>
-    <t>Staff Akuntansi Dian</t>
-  </si>
-  <si>
-    <t>192.168.141.122</t>
-  </si>
-  <si>
-    <t>Staff Mutu</t>
-  </si>
-  <si>
-    <t>192.168.141.121</t>
-  </si>
-  <si>
-    <t>PPI</t>
-  </si>
-  <si>
-    <t>192.168.141.136</t>
-  </si>
-  <si>
-    <t>SPV Perawat Pak Rizal</t>
-  </si>
-  <si>
-    <t>192.168.141.135</t>
-  </si>
-  <si>
-    <t>SPV Legal</t>
-  </si>
-  <si>
-    <t>SDM</t>
-  </si>
-  <si>
-    <t>192.168.141.133</t>
-  </si>
-  <si>
-    <t>Staff Diklat dan Pengembangan</t>
-  </si>
-  <si>
-    <t>192.168.141.131</t>
-  </si>
-  <si>
-    <t>Staff SDM Aldi</t>
-  </si>
-  <si>
-    <t>Staff Legal Fajar</t>
-  </si>
-  <si>
-    <t>192.168.141.130</t>
-  </si>
-  <si>
-    <t>SPV Teknologi Informasi</t>
-  </si>
-  <si>
-    <t>IT</t>
-  </si>
-  <si>
-    <t>192.168.142.20</t>
-  </si>
-  <si>
-    <t>Pengembangan Sistem Novit</t>
-  </si>
-  <si>
-    <t>192.168.142.88</t>
-  </si>
-  <si>
-    <t>Infrastruktur Iyan</t>
-  </si>
-  <si>
-    <t>192.168.142.12</t>
-  </si>
-  <si>
-    <t>Operasional IT Ibnu</t>
-  </si>
-  <si>
-    <t>192.168.142.22</t>
-  </si>
-  <si>
-    <t>Operasional IT Samuel</t>
-  </si>
-  <si>
-    <t>192.168.142.33</t>
-  </si>
-  <si>
-    <t>Nurstation Lt4 1</t>
-  </si>
-  <si>
-    <t>192.168.143.121</t>
-  </si>
-  <si>
-    <t>Nurstation Lt4 2</t>
-  </si>
-  <si>
-    <t>192.168.143.120</t>
-  </si>
-  <si>
-    <t>KI Ranap</t>
-  </si>
-  <si>
-    <t>192.168.143.126</t>
-  </si>
-  <si>
-    <t>Staff Casemix Via</t>
-  </si>
-  <si>
-    <t>Casemix</t>
-  </si>
-  <si>
-    <t>192.168.151.139</t>
-  </si>
-  <si>
-    <t>Staff Casemix Ranti</t>
-  </si>
-  <si>
-    <t>192.168.151.137</t>
-  </si>
-  <si>
-    <t>Staff Casemix Noval</t>
-  </si>
-  <si>
-    <t>192.168.151.140</t>
-  </si>
-  <si>
-    <t>Staff Casemix Adi</t>
-  </si>
-  <si>
-    <t>192.168.151.141</t>
-  </si>
-  <si>
-    <t>Staff Casemix Ryan</t>
-  </si>
-  <si>
-    <t>192.168.151.136</t>
-  </si>
-  <si>
-    <t>Staff Casemix Yudha</t>
-  </si>
-  <si>
-    <t>192.168.151.142</t>
-  </si>
-  <si>
-    <t>Staff Casemix Wahyu</t>
-  </si>
-  <si>
-    <t>192.168.151.143</t>
-  </si>
-  <si>
-    <t>Nurstation Lt5 1</t>
-  </si>
-  <si>
-    <t>192.168.151.121</t>
-  </si>
-  <si>
-    <t>Nurstation Lt5 2</t>
-  </si>
-  <si>
-    <t>192.168.151.120</t>
-  </si>
-  <si>
-    <t>Nurstation Lt5 3</t>
-  </si>
-  <si>
-    <t>192.168.151.122</t>
-  </si>
-  <si>
-    <t>Fisioterapi</t>
-  </si>
-  <si>
-    <t>192.168.141.134</t>
-  </si>
-  <si>
-    <t>IPSRS</t>
-  </si>
-  <si>
-    <t>Poli</t>
-  </si>
-  <si>
-    <t>Keuangan &amp; Akuntansi</t>
-  </si>
-  <si>
-    <t>Komite</t>
   </si>
 </sst>
 </file>
@@ -849,7 +849,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -872,16 +872,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1186,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1218,7 +1238,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1226,8 +1246,8 @@
       <c r="D2" s="1">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
+      <c r="E2" s="5" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1235,7 +1255,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1243,8 +1263,8 @@
       <c r="D3" s="1">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>9</v>
+      <c r="E3" s="5" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1252,7 +1272,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
@@ -1260,8 +1280,8 @@
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>11</v>
+      <c r="E4" s="5" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1269,7 +1289,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
@@ -1277,8 +1297,8 @@
       <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>13</v>
+      <c r="E5" s="5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1286,16 +1306,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>16</v>
+      <c r="E6" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1303,7 +1323,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
@@ -1312,7 +1332,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1320,7 +1340,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
@@ -1329,7 +1349,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1337,16 +1357,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D9" s="1">
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1354,16 +1374,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1371,16 +1391,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1388,16 +1408,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1405,16 +1425,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1">
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1422,16 +1442,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1439,16 +1459,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D15" s="1">
         <v>1</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1456,16 +1476,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D16" s="1">
         <v>1</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1473,16 +1493,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D17" s="1">
         <v>1</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>40</v>
+      <c r="E17" s="5" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1490,16 +1510,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D18" s="1">
         <v>1</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>42</v>
+      <c r="E18" s="5" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1507,16 +1527,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D19" s="1">
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1524,16 +1544,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D20" s="1">
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1541,16 +1561,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D21" s="1">
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1558,16 +1578,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D22" s="1">
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1575,16 +1595,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D23" s="1">
         <v>1</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1592,33 +1612,33 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D24" s="1">
         <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>57</v>
+      <c r="B25" s="4" t="s">
+        <v>259</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="D25" s="1">
-        <v>1</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1626,16 +1646,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D26" s="1">
         <v>1</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1643,16 +1663,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D27" s="1">
         <v>1</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1660,16 +1680,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>63</v>
+        <v>255</v>
       </c>
       <c r="D28" s="1">
         <v>1</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1677,16 +1697,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D29" s="1">
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1694,16 +1714,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1711,16 +1731,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D31" s="1">
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1728,16 +1748,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D32" s="1">
         <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1745,16 +1765,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="D33" s="1">
         <v>1</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1762,16 +1782,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="D34" s="1">
         <v>1</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1779,16 +1799,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D35" s="1">
         <v>1</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1796,16 +1816,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D36" s="1">
         <v>1</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1813,16 +1833,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D37" s="1">
         <v>1</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1830,16 +1850,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1847,16 +1867,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D39" s="1">
         <v>1</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1864,16 +1884,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>264</v>
+        <v>11</v>
       </c>
       <c r="D40" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1881,16 +1901,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="D41" s="1">
         <v>2</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1898,16 +1918,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>92</v>
+        <v>253</v>
       </c>
       <c r="D42" s="1">
         <v>2</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1915,16 +1935,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
       <c r="D43" s="1">
         <v>2</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1932,7 +1952,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>6</v>
@@ -1941,7 +1961,7 @@
         <v>2</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1949,7 +1969,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>6</v>
@@ -1958,7 +1978,7 @@
         <v>2</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1966,16 +1986,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>264</v>
+        <v>6</v>
       </c>
       <c r="D46" s="1">
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1983,16 +2003,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D47" s="1">
         <v>2</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -2000,16 +2020,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D48" s="1">
         <v>2</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -2017,16 +2037,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D49" s="1">
         <v>2</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -2034,16 +2054,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D50" s="1">
         <v>2</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -2051,16 +2071,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>92</v>
+        <v>256</v>
       </c>
       <c r="D51" s="1">
         <v>2</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -2068,16 +2088,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D52" s="1">
         <v>2</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -2085,16 +2105,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D53" s="1">
         <v>2</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -2102,16 +2122,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D54" s="1">
         <v>2</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -2119,16 +2139,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D55" s="1">
         <v>2</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -2136,16 +2156,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D56" s="1">
         <v>2</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -2153,16 +2173,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D57" s="1">
         <v>2</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -2170,16 +2190,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D58" s="1">
         <v>2</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -2187,16 +2207,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D59" s="1">
         <v>2</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -2204,16 +2224,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D60" s="1">
         <v>2</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -2221,16 +2241,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D61" s="1">
         <v>2</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -2238,16 +2258,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D62" s="1">
         <v>2</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -2255,16 +2275,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D63" s="1">
         <v>2</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -2272,16 +2292,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D64" s="1">
         <v>2</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -2289,16 +2309,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D65" s="1">
         <v>2</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -2306,16 +2326,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D66" s="1">
         <v>2</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -2323,16 +2343,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>143</v>
+        <v>86</v>
       </c>
       <c r="D67" s="1">
         <v>2</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -2340,16 +2360,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D68" s="1">
         <v>2</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -2357,16 +2377,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D69" s="1">
         <v>2</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2374,16 +2394,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D70" s="1">
         <v>2</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -2391,16 +2411,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D71" s="1">
         <v>2</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2408,16 +2428,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D72" s="1">
         <v>2</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -2425,16 +2445,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="D73" s="1">
         <v>2</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -2442,16 +2462,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D74" s="1">
         <v>2</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -2459,16 +2479,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D75" s="1">
         <v>2</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -2476,16 +2496,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D76" s="1">
         <v>2</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2493,16 +2513,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>92</v>
+        <v>155</v>
       </c>
       <c r="D77" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -2510,16 +2530,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>168</v>
+        <v>86</v>
       </c>
       <c r="D78" s="1">
         <v>3</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -2527,16 +2547,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D79" s="1">
         <v>3</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -2544,16 +2564,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>33</v>
+        <v>162</v>
       </c>
       <c r="D80" s="1">
         <v>3</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -2561,16 +2581,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>168</v>
+        <v>29</v>
       </c>
       <c r="D81" s="1">
         <v>3</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -2578,16 +2598,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="D82" s="1">
         <v>3</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -2595,16 +2615,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D83" s="1">
         <v>3</v>
       </c>
-      <c r="E83" s="1" t="s">
-        <v>180</v>
+      <c r="E83" s="3">
+        <v>192168133120</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -2612,16 +2632,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="D84" s="1">
         <v>3</v>
       </c>
-      <c r="E84" s="1" t="s">
-        <v>183</v>
+      <c r="E84" s="3">
+        <v>192168133121</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -2629,16 +2649,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D85" s="1">
         <v>3</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2646,16 +2666,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="D86" s="1">
         <v>3</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2663,16 +2683,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D87" s="1">
         <v>3</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -2680,16 +2700,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D88" s="1">
         <v>3</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -2697,16 +2717,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>265</v>
+        <v>179</v>
       </c>
       <c r="D89" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -2714,16 +2734,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D90" s="1">
         <v>4</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2731,16 +2751,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D91" s="1">
         <v>4</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -2748,16 +2768,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D92" s="1">
         <v>4</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -2765,16 +2785,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D93" s="1">
         <v>4</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -2782,16 +2802,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D94" s="1">
         <v>4</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2799,16 +2819,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D95" s="1">
         <v>4</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -2816,16 +2836,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="D96" s="1">
         <v>4</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
@@ -2833,16 +2853,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="D97" s="1">
         <v>4</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -2850,16 +2870,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="D98" s="1">
         <v>4</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
@@ -2867,16 +2887,16 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>187</v>
+        <v>258</v>
       </c>
       <c r="D99" s="1">
         <v>4</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -2884,16 +2904,16 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>216</v>
+        <v>179</v>
       </c>
       <c r="D100" s="1">
         <v>4</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
@@ -2901,16 +2921,16 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D101" s="1">
         <v>4</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>262</v>
+        <v>209</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
@@ -2918,16 +2938,16 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D102" s="1">
         <v>4</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -2935,16 +2955,16 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D103" s="1">
         <v>4</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -2952,16 +2972,16 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="D104" s="1">
         <v>4</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
@@ -2969,16 +2989,16 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D105" s="1">
         <v>4</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -2986,16 +3006,16 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D106" s="1">
         <v>4</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
@@ -3003,16 +3023,16 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D107" s="1">
         <v>4</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -3020,16 +3040,16 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D108" s="1">
         <v>4</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -3037,16 +3057,16 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="D109" s="1">
         <v>4</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
@@ -3054,16 +3074,16 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D110" s="1">
         <v>4</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
@@ -3071,16 +3091,16 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D111" s="1">
         <v>4</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
@@ -3088,16 +3108,16 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>241</v>
+        <v>179</v>
       </c>
       <c r="D112" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
@@ -3105,16 +3125,16 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D113" s="1">
         <v>5</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
@@ -3122,16 +3142,16 @@
         <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D114" s="1">
         <v>5</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
@@ -3139,16 +3159,16 @@
         <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D115" s="1">
         <v>5</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -3156,16 +3176,16 @@
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D116" s="1">
         <v>5</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
@@ -3173,16 +3193,16 @@
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D117" s="1">
         <v>5</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
@@ -3190,16 +3210,16 @@
         <v>117</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D118" s="1">
         <v>5</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
@@ -3207,16 +3227,16 @@
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
       <c r="D119" s="1">
         <v>5</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
@@ -3224,16 +3244,16 @@
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D120" s="1">
         <v>5</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
@@ -3241,16 +3261,33 @@
         <v>120</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D121" s="1">
         <v>5</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>260</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>121</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D122" s="1">
+        <v>5</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>